<commit_message>
Fix tests failing due to change of style writer
No semantic change to the test.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/StyleReferenceFiles/FillAtReservedPosition-MoveFill-Output.xlsx
+++ b/ClosedXML.Tests/Resource/Other/StyleReferenceFiles/FillAtReservedPosition-MoveFill-Output.xlsx
@@ -39,96 +39,67 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2 xr">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="2" x14ac:knownFonts="1">
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-      <x:scheme val="minor"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="5">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="darkGray">
-        <x:fgColor rgb="FF00B050"/>
-        <x:bgColor theme="0"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="lightGrid">
-        <x:fgColor rgb="FFFF0000"/>
-        <x:bgColor theme="0"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="4">
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="5">
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="1" borderId="0" xfId="0" applyFill="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="4">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="darkGray">
+        <fgColor rgb="FF00B050"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="lightGrid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </x:ext>
-    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </x:ext>
-  </x:extLst>
-</x:styleSheet>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -433,13 +404,10 @@
   </x:sheetPr>
   <x:dimension ref="A1:B1"/>
   <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <x:cols>
-    <x:col min="1" max="16384" width="9.140625" style="1" customWidth="1"/>
-  </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A1" s="3"/>
-      <x:c r="B1" s="4"/>
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="2"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>